<commit_message>
Scheduler v1.4: rebalance sample to 20% past-due, 30% tight, 50% relaxed
Both the in-app "Load sample" generator and the bundled
sample_mos.xlsx now produce 32 MOs with the requested mix:

  ~20% (6/32) have a delivery date already in the past — RED bars
                 on load, illustrating "always late" cases.

  ~24% (8/32) — 30% of the on-time ones — have due date == scheduled
                 end (zero slack). They start blue and turn yellow as
                 soon as the planner moves them forward by any amount.

  ~56% (18/32) have 5–18 days of slack between end and due date,
                 so they remain blue across most reasonable scenarios.

Categories are shuffled so the three classes are interleaved across
work centers and MO IDs.

https://claude.ai/code/session_01DrpP7pDJyV87w2ZB2tFERq
</commit_message>
<xml_diff>
--- a/production-scenario-scheduler/sample_mos.xlsx
+++ b/production-scenario-scheduler/sample_mos.xlsx
@@ -493,10 +493,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>504</v>
+        <v>160</v>
       </c>
       <c r="D2" t="n">
-        <v>8</v>
+        <v>30</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -509,13 +509,13 @@
         </is>
       </c>
       <c r="G2" s="2" t="n">
-        <v>46151</v>
+        <v>46182</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46156</v>
+        <v>46173</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>46156</v>
+        <v>46176</v>
       </c>
     </row>
     <row r="3">
@@ -530,10 +530,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>940</v>
+        <v>714</v>
       </c>
       <c r="D3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -546,13 +546,13 @@
         </is>
       </c>
       <c r="G3" s="2" t="n">
-        <v>46149</v>
+        <v>46171</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46156</v>
+        <v>46163</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>46156</v>
+        <v>46163</v>
       </c>
     </row>
     <row r="4">
@@ -567,10 +567,10 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>474</v>
+        <v>551</v>
       </c>
       <c r="D4" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -583,13 +583,13 @@
         </is>
       </c>
       <c r="G4" s="2" t="n">
-        <v>46153</v>
+        <v>46181</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46156</v>
+        <v>46171</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>46156</v>
+        <v>46171</v>
       </c>
     </row>
     <row r="5">
@@ -604,10 +604,10 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>619</v>
+        <v>300</v>
       </c>
       <c r="D5" t="n">
-        <v>5</v>
+        <v>22</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -620,13 +620,13 @@
         </is>
       </c>
       <c r="G5" s="2" t="n">
-        <v>46153</v>
+        <v>46172</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46156</v>
+        <v>46170</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>46156</v>
+        <v>46172</v>
       </c>
     </row>
     <row r="6">
@@ -641,10 +641,10 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>188</v>
+        <v>755</v>
       </c>
       <c r="D6" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -657,13 +657,13 @@
         </is>
       </c>
       <c r="G6" s="2" t="n">
-        <v>46167</v>
+        <v>46149</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46166</v>
+        <v>46156</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>46166</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="7">
@@ -678,10 +678,10 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>171</v>
+        <v>104</v>
       </c>
       <c r="D7" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -694,13 +694,13 @@
         </is>
       </c>
       <c r="G7" s="2" t="n">
-        <v>46174</v>
+        <v>46165</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46171</v>
+        <v>46164</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>46173</v>
+        <v>46165</v>
       </c>
     </row>
     <row r="8">
@@ -715,10 +715,10 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>664</v>
+        <v>770</v>
       </c>
       <c r="D8" t="n">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -731,13 +731,13 @@
         </is>
       </c>
       <c r="G8" s="2" t="n">
-        <v>46168</v>
+        <v>46174</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46167</v>
+        <v>46159</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>46167</v>
+        <v>46162</v>
       </c>
     </row>
     <row r="9">
@@ -752,10 +752,10 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>946</v>
+        <v>664</v>
       </c>
       <c r="D9" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -768,13 +768,13 @@
         </is>
       </c>
       <c r="G9" s="2" t="n">
-        <v>46174</v>
+        <v>46164</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46173</v>
+        <v>46163</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>46173</v>
+        <v>46164</v>
       </c>
     </row>
     <row r="10">
@@ -789,10 +789,10 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>328</v>
+        <v>360</v>
       </c>
       <c r="D10" t="n">
-        <v>7</v>
+        <v>30</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -805,13 +805,13 @@
         </is>
       </c>
       <c r="G10" s="2" t="n">
-        <v>46179</v>
+        <v>46178</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46178</v>
+        <v>46159</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>46178</v>
+        <v>46162</v>
       </c>
     </row>
     <row r="11">
@@ -826,10 +826,10 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>696</v>
+        <v>625</v>
       </c>
       <c r="D11" t="n">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -842,13 +842,13 @@
         </is>
       </c>
       <c r="G11" s="2" t="n">
-        <v>46181</v>
+        <v>46149</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46178</v>
+        <v>46156</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>46180</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="12">
@@ -863,10 +863,10 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>699</v>
+        <v>171</v>
       </c>
       <c r="D12" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -879,13 +879,13 @@
         </is>
       </c>
       <c r="G12" s="2" t="n">
-        <v>46162</v>
+        <v>46158</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46159</v>
+        <v>46157</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>46161</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="13">
@@ -900,10 +900,10 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>326</v>
+        <v>210</v>
       </c>
       <c r="D13" t="n">
-        <v>5</v>
+        <v>22</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -916,13 +916,13 @@
         </is>
       </c>
       <c r="G13" s="2" t="n">
-        <v>46173</v>
+        <v>46171</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46172</v>
+        <v>46169</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>46172</v>
+        <v>46171</v>
       </c>
     </row>
     <row r="14">
@@ -937,10 +937,10 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>979</v>
+        <v>966</v>
       </c>
       <c r="D14" t="n">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -953,13 +953,13 @@
         </is>
       </c>
       <c r="G14" s="2" t="n">
-        <v>46162</v>
+        <v>46159</v>
       </c>
       <c r="H14" s="2" t="n">
+        <v>46158</v>
+      </c>
+      <c r="I14" s="2" t="n">
         <v>46159</v>
-      </c>
-      <c r="I14" s="2" t="n">
-        <v>46161</v>
       </c>
     </row>
     <row r="15">
@@ -974,7 +974,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>529</v>
+        <v>168</v>
       </c>
       <c r="D15" t="n">
         <v>13</v>
@@ -990,13 +990,13 @@
         </is>
       </c>
       <c r="G15" s="2" t="n">
-        <v>46165</v>
+        <v>46152</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46163</v>
+        <v>46156</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>46164</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="16">
@@ -1011,10 +1011,10 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>220</v>
+        <v>318</v>
       </c>
       <c r="D16" t="n">
-        <v>21</v>
+        <v>4</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -1027,13 +1027,13 @@
         </is>
       </c>
       <c r="G16" s="2" t="n">
-        <v>46165</v>
+        <v>46146</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46162</v>
+        <v>46156</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>46164</v>
+        <v>46156</v>
       </c>
     </row>
     <row r="17">
@@ -1048,10 +1048,10 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>673</v>
+        <v>581</v>
       </c>
       <c r="D17" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -1064,13 +1064,13 @@
         </is>
       </c>
       <c r="G17" s="2" t="n">
-        <v>46179</v>
+        <v>46158</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46177</v>
+        <v>46157</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>46178</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="18">
@@ -1085,10 +1085,10 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>285</v>
+        <v>174</v>
       </c>
       <c r="D18" t="n">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -1101,13 +1101,13 @@
         </is>
       </c>
       <c r="G18" s="2" t="n">
-        <v>46187</v>
+        <v>46181</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46183</v>
+        <v>46169</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>46186</v>
+        <v>46170</v>
       </c>
     </row>
     <row r="19">
@@ -1122,7 +1122,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>684</v>
+        <v>897</v>
       </c>
       <c r="D19" t="n">
         <v>22</v>
@@ -1138,13 +1138,13 @@
         </is>
       </c>
       <c r="G19" s="2" t="n">
-        <v>46164</v>
+        <v>46149</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46161</v>
+        <v>46156</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>46163</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="20">
@@ -1159,10 +1159,10 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>481</v>
+        <v>189</v>
       </c>
       <c r="D20" t="n">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -1175,13 +1175,13 @@
         </is>
       </c>
       <c r="G20" s="2" t="n">
-        <v>46181</v>
+        <v>46178</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46179</v>
+        <v>46165</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>46180</v>
+        <v>46168</v>
       </c>
     </row>
     <row r="21">
@@ -1196,10 +1196,10 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>829</v>
+        <v>519</v>
       </c>
       <c r="D21" t="n">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -1212,13 +1212,13 @@
         </is>
       </c>
       <c r="G21" s="2" t="n">
-        <v>46164</v>
+        <v>46173</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46161</v>
+        <v>46167</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>46163</v>
+        <v>46168</v>
       </c>
     </row>
     <row r="22">
@@ -1233,10 +1233,10 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>161</v>
+        <v>352</v>
       </c>
       <c r="D22" t="n">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -1249,13 +1249,13 @@
         </is>
       </c>
       <c r="G22" s="2" t="n">
-        <v>46163</v>
+        <v>46170</v>
       </c>
       <c r="H22" s="2" t="n">
         <v>46160</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
     </row>
     <row r="23">
@@ -1270,10 +1270,10 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>608</v>
+        <v>111</v>
       </c>
       <c r="D23" t="n">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -1286,13 +1286,13 @@
         </is>
       </c>
       <c r="G23" s="2" t="n">
-        <v>46180</v>
+        <v>46147</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46178</v>
+        <v>46156</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>46179</v>
+        <v>46159</v>
       </c>
     </row>
     <row r="24">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>537</v>
+        <v>916</v>
       </c>
       <c r="D24" t="n">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -1323,13 +1323,13 @@
         </is>
       </c>
       <c r="G24" s="2" t="n">
-        <v>46182</v>
+        <v>46164</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46179</v>
+        <v>46164</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>46181</v>
+        <v>46164</v>
       </c>
     </row>
     <row r="25">
@@ -1344,10 +1344,10 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>576</v>
+        <v>672</v>
       </c>
       <c r="D25" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -1360,13 +1360,13 @@
         </is>
       </c>
       <c r="G25" s="2" t="n">
-        <v>46185</v>
+        <v>46179</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46183</v>
+        <v>46162</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>46184</v>
+        <v>46164</v>
       </c>
     </row>
     <row r="26">
@@ -1381,10 +1381,10 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>470</v>
+        <v>295</v>
       </c>
       <c r="D26" t="n">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -1397,13 +1397,13 @@
         </is>
       </c>
       <c r="G26" s="2" t="n">
-        <v>46179</v>
+        <v>46185</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46176</v>
+        <v>46171</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>46178</v>
+        <v>46172</v>
       </c>
     </row>
     <row r="27">
@@ -1418,10 +1418,10 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>913</v>
+        <v>759</v>
       </c>
       <c r="D27" t="n">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1434,13 +1434,13 @@
         </is>
       </c>
       <c r="G27" s="2" t="n">
-        <v>46170</v>
+        <v>46175</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46168</v>
+        <v>46161</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>46169</v>
+        <v>46164</v>
       </c>
     </row>
     <row r="28">
@@ -1455,10 +1455,10 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>898</v>
+        <v>530</v>
       </c>
       <c r="D28" t="n">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1471,13 +1471,13 @@
         </is>
       </c>
       <c r="G28" s="2" t="n">
-        <v>46166</v>
+        <v>46172</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46162</v>
+        <v>46160</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>46165</v>
+        <v>46161</v>
       </c>
     </row>
     <row r="29">
@@ -1492,10 +1492,10 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>688</v>
+        <v>985</v>
       </c>
       <c r="D29" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1508,13 +1508,13 @@
         </is>
       </c>
       <c r="G29" s="2" t="n">
-        <v>46168</v>
+        <v>46167</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46167</v>
+        <v>46157</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>46167</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="30">
@@ -1529,10 +1529,10 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>606</v>
+        <v>120</v>
       </c>
       <c r="D30" t="n">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1545,13 +1545,13 @@
         </is>
       </c>
       <c r="G30" s="2" t="n">
-        <v>46170</v>
+        <v>46187</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46167</v>
+        <v>46175</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>46169</v>
+        <v>46178</v>
       </c>
     </row>
     <row r="31">
@@ -1566,10 +1566,10 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>559</v>
+        <v>974</v>
       </c>
       <c r="D31" t="n">
-        <v>27</v>
+        <v>10</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1582,13 +1582,13 @@
         </is>
       </c>
       <c r="G31" s="2" t="n">
-        <v>46171</v>
+        <v>46174</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46167</v>
+        <v>46162</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>46170</v>
+        <v>46163</v>
       </c>
     </row>
     <row r="32">
@@ -1603,7 +1603,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>174</v>
+        <v>143</v>
       </c>
       <c r="D32" t="n">
         <v>23</v>
@@ -1619,13 +1619,13 @@
         </is>
       </c>
       <c r="G32" s="2" t="n">
-        <v>46170</v>
+        <v>46183</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46167</v>
+        <v>46175</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>46169</v>
+        <v>46177</v>
       </c>
     </row>
     <row r="33">
@@ -1640,10 +1640,10 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>528</v>
+        <v>364</v>
       </c>
       <c r="D33" t="n">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1656,10 +1656,10 @@
         </is>
       </c>
       <c r="G33" s="2" t="n">
-        <v>46164</v>
+        <v>46175</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>46161</v>
+        <v>46163</v>
       </c>
       <c r="I33" s="2" t="n">
         <v>46163</v>

</xml_diff>